<commit_message>
Fix duplicate titles on Labor Market and Pathway Mapping pages
</commit_message>
<xml_diff>
--- a/JA_BizTown_RFP_Clarification_Questions.xlsx
+++ b/JA_BizTown_RFP_Clarification_Questions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Satya Siva Parasa\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Venkata\JA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516D5A1B-C43D-4BB1-B8DC-69A023900786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{132296BF-62B1-4167-902B-DC1F6BE02DC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="18000" windowHeight="10433" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clarification Questions" sheetId="1" r:id="rId1"/>

</xml_diff>